<commit_message>
Stage 8 review fixes: HO-007
</commit_message>
<xml_diff>
--- a/output/archive/Tarnovell_Group/Integration/SharePoint/2026/SharePoint_Migration_Tracker_2026-09.xlsx
+++ b/output/archive/Tarnovell_Group/Integration/SharePoint/2026/SharePoint_Migration_Tracker_2026-09.xlsx
@@ -140,21 +140,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Sofia Lindervik</author>
-  </authors>
-  <commentList>
-    <comment ref="F3" authorId="0" shapeId="0">
-      <text>
-        <t>Ownership for Chem-Shared is being traced through the leaver list from HR. Do not move the folders until this is closed.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -456,7 +441,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SharePoint migration tracker - September 2026</t>
+          <t>Tarnovell Bioscience Group | SharePoint migration tracker - September 2026</t>
         </is>
       </c>
     </row>
@@ -517,7 +502,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>A task is closed only when the sign-off named on the Share sheet is recorded. Nothing is closed because a copy has completed.</t>
+          <t>Close a migration task only when inventory, permission mapping, ownership checks and any exception sign-off are recorded under Procedure v2. A completed copy is insufficient.</t>
         </is>
       </c>
     </row>
@@ -557,12 +542,12 @@
       </c>
       <c r="B1" s="3" t="inlineStr">
         <is>
-          <t>Share root</t>
+          <t>Share scope</t>
         </is>
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
-          <t>Archive root</t>
+          <t>Archive-root plan</t>
         </is>
       </c>
       <c r="D1" s="3" t="inlineStr">
@@ -572,7 +557,7 @@
       </c>
       <c r="E1" s="3" t="inlineStr">
         <is>
-          <t>Owner confirmed</t>
+          <t>Ownership check</t>
         </is>
       </c>
       <c r="F1" s="3" t="inlineStr">
@@ -599,12 +584,12 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>VM-Ledger</t>
+          <t>Historical chemistry records; inventory reference pending</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>/Archive/A/Ledger</t>
+          <t>Preserve separate local archive root; mapping pending</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -614,22 +599,22 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Confirmation required</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Checked</t>
+          <t>Ownership check required</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Closed</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Original notebooks scanned and linked</t>
+          <t>Acceptance evidence pending: inventory, permissions and ownership; preserve original scientific records</t>
         </is>
       </c>
     </row>
@@ -641,12 +626,12 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Chem-Shared</t>
+          <t>Chemistry shared records; inventory reference pending</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>/Archive/A/Chem</t>
+          <t>Preserve separate local archive root; mapping pending</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -656,12 +641,12 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Confirmation required</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Ownership check required</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -671,7 +656,7 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Two leaver folders with no active owner</t>
+          <t>Acceptance evidence pending: inventory, permissions and ownership; preserve original scientific records</t>
         </is>
       </c>
     </row>
@@ -683,12 +668,12 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Screening-Data</t>
+          <t>Screening records; inventory reference pending</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>/Archive/B/Screen</t>
+          <t>Preserve separate local archive root; mapping pending</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -698,22 +683,22 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Confirmation required</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Checked</t>
+          <t>Ownership check required</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Closed</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Plate-reader exports kept in original format</t>
+          <t>Acceptance evidence pending: inventory, permissions and ownership; preserve original scientific records</t>
         </is>
       </c>
     </row>
@@ -725,12 +710,12 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Assay-Protocols</t>
+          <t>Assay protocols; inventory reference pending</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>/Archive/B/Protocols</t>
+          <t>Preserve separate local archive root; mapping pending</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -740,12 +725,12 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Confirmation required</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Ownership check required</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -755,7 +740,7 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Owner to be confirmed by the biology lead</t>
+          <t>Acceptance evidence pending: inventory, permissions and ownership; preserve original scientific records</t>
         </is>
       </c>
     </row>
@@ -767,12 +752,12 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Bioanalysis-Raw</t>
+          <t>Bioanalysis raw records; inventory reference pending</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>/Archive/C/Raw</t>
+          <t>Preserve separate local archive root; mapping pending</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -782,22 +767,22 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Confirmation required</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Checked</t>
+          <t>Ownership check required</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Closed</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Raw acquisition files retained with audit trail</t>
+          <t>Acceptance evidence pending: inventory, permissions and ownership; preserve original scientific records</t>
         </is>
       </c>
     </row>
@@ -809,12 +794,12 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Report-Drafts</t>
+          <t>Draft and superseded reports; inventory reference pending</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>/Archive/C/Drafts</t>
+          <t>Preserve separate local archive root; mapping pending</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -824,12 +809,12 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Confirmation required</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Ownership check required</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -839,7 +824,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Draft reports mixed with superseded versions</t>
+          <t>Acceptance evidence pending: inventory, permissions and ownership; preserve original scientific records</t>
         </is>
       </c>
     </row>
@@ -851,12 +836,12 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Compute-Projects</t>
+          <t>Computational project records; inventory reference pending</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>/Archive/D/Projects</t>
+          <t>Preserve separate local archive root; mapping pending</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -866,12 +851,12 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Confirmation required</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Not applicable</t>
+          <t>Ownership check required</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -881,7 +866,7 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Permissions review pending</t>
+          <t>Acceptance evidence pending: inventory, permissions and ownership; preserve original scientific records</t>
         </is>
       </c>
     </row>
@@ -893,12 +878,12 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Stability-Chambers</t>
+          <t>Stability records; inventory reference pending</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>/Archive/E/Stability</t>
+          <t>Preserve separate local archive root; mapping pending</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -908,12 +893,12 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Confirmation required</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Ownership check required</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -923,7 +908,7 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Chamber logs being matched to studies</t>
+          <t>Acceptance evidence pending: inventory, permissions and ownership; preserve original scientific records</t>
         </is>
       </c>
     </row>
@@ -935,12 +920,12 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Formulation-Share</t>
+          <t>Formulation records; inventory reference pending</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>/Archive/F/Formulation</t>
+          <t>Preserve separate local archive root; mapping pending</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -950,12 +935,12 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Confirmation required</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Checked</t>
+          <t>Ownership check required</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -965,7 +950,7 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Migration nearly complete; permission sweep outstanding</t>
+          <t>Acceptance evidence pending: inventory, permissions and ownership; preserve original scientific records</t>
         </is>
       </c>
     </row>
@@ -977,27 +962,27 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Osterquill-Legacy</t>
+          <t>Osterquill local archive (planning only)</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Not migrated</t>
+          <t>No migration before completion</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Held apart</t>
+          <t>Hold apart after completion pending access and QA mapping</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Not applicable</t>
+          <t>Pending post-completion review</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Not applicable</t>
+          <t>Pending post-completion review</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -1007,14 +992,13 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Access and QA mapping before any move; completion 1 October 2026</t>
+          <t>Planned completion 1 October 2026; not yet a group firm at this snapshot</t>
         </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -1024,7 +1008,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1073,7 +1057,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Confirm owner of Assay-Protocols (B)</t>
+          <t>Confirm ownership of B assay protocol records</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -1083,12 +1067,12 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>17/10/2026</t>
+          <t>To be agreed</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Move of B protocols</t>
+          <t>Move of B protocol records</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -1103,7 +1087,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Trace owners of two leaver folders in Chem-Shared (A)</t>
+          <t>Confirm ownership of A chemistry leaver folders</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -1113,12 +1097,12 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>24/10/2026</t>
+          <t>To be agreed</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Move of A chemistry share</t>
+          <t>Move of A chemistry records</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -1133,7 +1117,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Review draft reports in Report-Drafts (C) against superseded versions</t>
+          <t>Review C draft reports against superseded versions</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -1143,7 +1127,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>31/10/2026</t>
+          <t>To be agreed</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -1163,7 +1147,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Permission sweep on Formulation-Share (F)</t>
+          <t>Complete F permission mapping and acceptance checks</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -1173,7 +1157,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>10/10/2026</t>
+          <t>To be agreed</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -1193,7 +1177,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Match stability chamber logs to studies (E)</t>
+          <t>Confirm E stability record retention and ownership</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -1203,7 +1187,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>31/10/2026</t>
+          <t>To be agreed</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -1223,25 +1207,55 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
+          <t>Confirm D computational share permissions</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>D site leadership</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>To be agreed</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>D migration acceptance</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
           <t>Osterquill access and QA mapping plan</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Yasmin Farhat</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>Before 1 October 2026 completion</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>G onboarding</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>Planning</t>
         </is>
@@ -1259,7 +1273,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1287,83 +1301,15 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>09/02/2026</t>
+          <t>25/09/2026</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Tracker created from the approved migration procedure; firms A-F listed</t>
+          <t>September snapshot: A-F acceptance checks remain open; Osterquill listed for pre-completion planning only</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Sofia Lindervik</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>03/04/2026</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Share inventories for A and B added; owners requested for leaver folders</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Sofia Lindervik</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>18/06/2026</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Retention decisions recorded for A-C; original scientific records retained</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Sofia Lindervik</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>21/07/2026</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Exception for C draft reports raised with Group Quality</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Sofia Lindervik</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>25/09/2026</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>September snapshot; open items moved to the Open items sheet</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Sofia Lindervik</t>
         </is>

</xml_diff>